<commit_message>
Move the Safety and Trust Engine readme into Agentic AI.
</commit_message>
<xml_diff>
--- a/data/links.xlsx
+++ b/data/links.xlsx
@@ -5720,7 +5720,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>Agentic AI</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Computer_Vision/safety-trust-engine/README_es.md</t>
+          <t>Agentic_AI/safety-trust-engine/README_es.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the latest Spanish videos and the README copies that were missing.
</commit_message>
<xml_diff>
--- a/data/links.xlsx
+++ b/data/links.xlsx
@@ -3177,7 +3177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5949,6 +5949,80 @@
       <c r="G80" t="inlineStr">
         <is>
           <t>OpenAI/DotNet_ML/README_es.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MLOPS</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>LLMOps: TurboQuant explicado: comprimir la KV cache de un LLM a 3,5 bits sin perder calidad</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>En video recorremos veremos la teoria y tecnologia detras de Turboquant , esta es la parte primera de 2 Videos</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://youtu.be/N2NGVO2aGZ8</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Added from the YouTube channel. This video was not in the CSV. | The description links to GitHub, but the README file could not be downloaded.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>https://github.com/olonok69/ML_TurboQuant</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>MLOPS/ML_TurboQuant/README_es.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Agentic AI</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Vibe Coding: Curso Claude Code Parte 2, la metodología de 11 etapas y el grafo de conocimiento</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Segunda y última entrega del curso de Claude Code en español. Las partes 2 y 3 van en un único vídeo porque cuentan la misma historia: cómo se trabaja de verdad con un agente en un proyecto en producción, y qué se construye encima cuando la memoria del proyecto se vuelve consultable.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://youtu.be/rUudW1oB8co</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Added from the YouTube channel. This video was not in the CSV. | The description links to GitHub, but the README file could not be downloaded.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>https://github.com/olonok69/claude_code_ml_engineer</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Agentic_AI/claude_code_ml_engineer/README_es.md</t>
         </is>
       </c>
     </row>

</xml_diff>